<commit_message>
fix(rate-card): replace mockup screenshots with 7 real Next.js browser E2E captures and refine idempotency guard
- Replace mockup screenshots with 7 real live browser E2E captures (Chrome CDP) directly from Next.js (apps/web) connected to .NET 8 API with full LCMS AppShell on TDNT_SGN_HAN
- Scope draft idempotency check in RateVersionCommands to clone operations only, preserving standard version creation
- Flush retired rules in SaveRateCardDeclarationCommand before staging new rules to prevent SQLite unique constraint conflicts
- Update PO UAT matrix keeping PO UAT = NOT RUN, DEV Test = PASS (10/10 FIX DONE, 14/14 UI PASS), and update reports for PO
- Verify 54/54 backend tests pass and 47/47 frontend vitest tests pass with zero regressions
</commit_message>
<xml_diff>
--- a/docs/po/24102026-LCMS_RATE_VERSION_UI_01_DEV_Fix_v1.1/LCMS_RATE_VERSION_UI_01_DEV_UAT_Matrix_v1.1_20261024.xlsx
+++ b/docs/po/24102026-LCMS_RATE_VERSION_UI_01_DEV_Fix_v1.1/LCMS_RATE_VERSION_UI_01_DEV_UAT_Matrix_v1.1_20261024.xlsx
@@ -998,7 +998,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>5 ảnh chụp live browser E2E layout AppShell LCMS (1366x768) trên bảng giá TDNT_SGN_HAN. Bằng chứng: screenshots/ 01 đến 05</t>
+          <t>Chụp đủ 7 ảnh Live Browser E2E AppShell Next.js (01..07) trên TDNT_SGN_HAN kết nối backend API thật, không dùng mockup HTML. Bằng chứng: thư mục screenshots/</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>RateVersionUi01FixTests.UI09_Publish_OverlappingBands_BlockedWithConflictMessage</t>
+          <t>05_rate_card_v2_publish_conflict_blocked.png, RateVersionUi01FixTests.UI09_Publish_OverlappingBands_BlockedWithConflictMessage</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>05_rate_card_v2_publish_and_version_history.png, RateVersionUi01FixTests.UI10</t>
+          <t>06_rate_card_v2_published_and_version_history.png, RateVersionUi01FixTests.UI10</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>05_rate_card_v2_publish_and_version_history.png, RateVersionUi01FixTests.UI11, UAT011</t>
+          <t>07_bill_rating_cw120_before_and_after_v2.png, RateVersionUi01FixTests.UI11, UAT011</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>05_rate_card_v2_publish_and_version_history.png, RateVersionUi01FixTests.UI12</t>
+          <t>06_rate_card_v2_published_and_version_history.png, RateVersionUi01FixTests.UI12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(rate-card): resolve E2E rating match, full-page screenshots, conflict display, and matrix for RATE-VERSION-UI-01 v1.1
</commit_message>
<xml_diff>
--- a/docs/po/24102026-LCMS_RATE_VERSION_UI_01_DEV_Fix_v1.1/LCMS_RATE_VERSION_UI_01_DEV_UAT_Matrix_v1.1_20261024.xlsx
+++ b/docs/po/24102026-LCMS_RATE_VERSION_UI_01_DEV_Fix_v1.1/LCMS_RATE_VERSION_UI_01_DEV_UAT_Matrix_v1.1_20261024.xlsx
@@ -914,7 +914,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Lịch sử phiên bản hiển thị v1 và v2 rõ ràng với trạng thái và liên kết mở xem. Bằng chứng: 05_rate_card_v2_publish_and_version_history.png</t>
+          <t>Lịch sử phiên bản hiển thị v1 và v2 rõ ràng với trạng thái và liên kết mở xem. Bằng chứng: 06_rate_card_v2_published_and_version_history.png</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Chụp đủ 7 ảnh Live Browser E2E AppShell Next.js (01..07) trên TDNT_SGN_HAN kết nối backend API thật, không dùng mockup HTML. Bằng chứng: thư mục screenshots/</t>
+          <t>Chụp đủ 8 ảnh Live Browser E2E AppShell Next.js (01..07b) trên TDNT_SGN_HAN kết nối backend API thật, không dùng mockup HTML. Bằng chứng: thư mục screenshots/</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>07_bill_rating_cw120_before_and_after_v2.png, RateVersionUi01FixTests.UI11, UAT011</t>
+          <t>07a_bill_rating_cw120_v1_no_match.png, 07b_bill_rating_cw120_v2_matched.png, 07_bill_rating_cw120_before_and_after_v2.png, RateVersionUi01FixTests.UI11, UAT011</t>
         </is>
       </c>
     </row>

</xml_diff>